<commit_message>
Add nutrition safety collapsible + update hazard log to v0.4
- Collapsible 'Consult your doctor' safety check on nutrition page listing
  conditions where dietary changes may be unsafe (diabetes, eating disorders,
  kidney disease, heart failure, warfarin, underweight, pregnancy)
- H04 controls updated: deficit cap + condition cautions now documented
- H04 open action marked complete
- Excel hazard log regenerated with v0.4 data (H01, H04, open actions, changelog)
- All email addresses confirmed as hello@jointjourney.org
</commit_message>
<xml_diff>
--- a/docs/clinical-safety/Joint Journey - Hazard Log (DCB0129).xlsx
+++ b/docs/clinical-safety/Joint Journey - Hazard Log (DCB0129).xlsx
@@ -57,13 +57,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF9800"/>
+      <color rgb="004CAF50"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="004CAF50"/>
+      <color rgb="00FF9800"/>
       <sz val="11"/>
     </font>
     <font>
@@ -108,12 +108,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
-        <bgColor rgb="00FFF8E1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E8F5E9"/>
         <bgColor rgb="00E8F5E9"/>
       </patternFill>
@@ -122,6 +116,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F5F5F5"/>
         <bgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+        <bgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
   </fills>
@@ -151,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,19 +167,16 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -710,26 +707,26 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>"Stop if sharp pain" guidance; "hold onto something sturdy"; "talk to your GP before starting"; gentle/standard/active levelling; warm-up instructions. Pre-exercise safety check collapsible (v0.2).</t>
+          <t>"Stop if sharp pain" guidance; "hold onto something sturdy"; "talk to your GP before starting"; gentle/standard/active levelling; warm-up instructions. Pre-exercise safety check collapsible (v0.2). PAR-Q-style safety screening questionnaire during onboarding (v0.4): heart/lung, balance/falls, GP-restricted exercise. Flagged users see persistent caution banner on exercise page.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Formal pre-start safety screening questionnaire; video demonstrations of correct form.</t>
+          <t>Video demonstrations of correct form.</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Partial — pre-exercise safety check live; formal questionnaire still to add.</t>
+          <t>Implemented (v0.4) — screening questionnaire + pre-exercise safety check live.</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -784,7 +781,7 @@
       <c r="K9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="L9" s="8" t="n">
+      <c r="L9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -825,7 +822,7 @@
       <c r="F10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="8" t="n">
         <v>6</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -844,7 +841,7 @@
       <c r="K10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="L10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -885,17 +882,17 @@
       <c r="F11" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="8" t="n">
         <v>6</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Presented as general guidance; estimates noted as approximate.</t>
+          <t>Presented as general guidance; estimates noted as approximate. Deficit only applied when BMI indicates weight to lose; capped at safe maximum (300–500 kcal/day); never below absolute calorie floor. Collapsible "Consult your doctor" safety check on nutrition page (v0.4): diabetes, eating disorders, kidney disease, heart failure, warfarin, underweight, pregnancy.</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Floor on minimum calories; signpost to GP/dietitian; exclude/caution for low BMI.</t>
+          <t>None outstanding — core controls in place.</t>
         </is>
       </c>
       <c r="J11" s="7" t="n">
@@ -904,12 +901,12 @@
       <c r="K11" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="L11" s="8" t="n">
+      <c r="L11" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>OPEN — min-calorie floor + condition cautions still to implement.</t>
+          <t>Implemented (v0.4) — deficit cap + condition cautions live.</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -964,7 +961,7 @@
       <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="L12" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M12" s="4" t="inlineStr">
@@ -1005,7 +1002,7 @@
       <c r="F13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -1024,7 +1021,7 @@
       <c r="K13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L13" s="8" t="n">
+      <c r="L13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
@@ -1065,7 +1062,7 @@
       <c r="F14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="8" t="n">
         <v>6</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1084,7 +1081,7 @@
       <c r="K14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="8" t="n">
+      <c r="L14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -1125,7 +1122,7 @@
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="8" t="n">
         <v>6</v>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1144,7 +1141,7 @@
       <c r="K15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L15" s="8" t="n">
+      <c r="L15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M15" s="7" t="inlineStr">
@@ -1185,7 +1182,7 @@
       <c r="F16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="6" t="n">
         <v>4</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1204,7 +1201,7 @@
       <c r="K16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="L16" s="8" t="n">
+      <c r="L16" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -1245,7 +1242,7 @@
       <c r="F17" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1264,7 +1261,7 @@
       <c r="K17" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="L17" s="8" t="n">
+      <c r="L17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M17" s="7" t="inlineStr">
@@ -1421,17 +1418,17 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Pre-exercise safety check (H01).</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Pre-exercise safety screening (H01).</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>v0.2 — safety check live; formal screening questionnaire still to add.</t>
+          <t>v0.4 — PAR-Q-style screening questionnaire in onboarding + caution banner on exercise page. Pre-exercise safety check also live (v0.2).</t>
         </is>
       </c>
     </row>
@@ -1455,17 +1452,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Minimum-calorie floor + condition cautions (H04).</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>Nutrition safety controls (H04).</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Implement in the nutrition/weight section of the app.</t>
+          <t>v0.4 — Deficit capped at 300–500 kcal/day, only applied when BMI indicates weight to lose. "Consult your doctor" collapsible on nutrition page.</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1472,7 @@
           <t>WCAG 2.1 AA accessibility pass (H08).</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1492,7 +1489,7 @@
           <t>Clinical advisory board review and sign-off (H01–H10).</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1509,7 +1506,7 @@
           <t>Formal CSO sign-off of this log (bump to v1.0).</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1535,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1570,7 +1567,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1580,39 +1577,56 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>CSO registered (action closed). Manufacturer updated to Elan Health Ltd (17347255). DPIA cross-reference added to H07 (action closed). H09 and H10 added. Excel hazard log generator created.</t>
+          <t>Safety screening questionnaire added to onboarding (PAR-Q-style: heart/lung, balance/falls, exercise restriction). Caution banner on exercise page for flagged users. "Consult your doctor" collapsible added to nutrition page. H01 residual risk reduced to 2×2=4. H04 controls updated, action closed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>18/07/2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>In-app safety controls implemented: persistent "When to seek help" header control (H02), crisis signposting including Samaritans (H05), pre-exercise safety check (H01).</t>
+          <t>CSO registered (action closed). Manufacturer updated to Elan Health Ltd (17347255). DPIA cross-reference added to H07 (action closed). H09 and H10 added. Excel hazard log generator created.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>In-app safety controls implemented: persistent "When to seek help" header control (H02), crisis signposting including Samaritans (H05), pre-exercise safety check (H01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>29/06/2026</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Initial draft. H01–H08 identified. First-pass risk ratings.</t>
         </is>

</xml_diff>